<commit_message>
Fixed BOM and Employee Leave Details in HRM test scenarios
Fixed BOM and Employee Leave Details in HRM test scenarios
</commit_message>
<xml_diff>
--- a/testdata/PMF - Scenarios.xlsx
+++ b/testdata/PMF - Scenarios.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="390" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="417" uniqueCount="96">
   <si>
     <t>Production Order - All Inside</t>
   </si>
@@ -306,6 +306,15 @@
   </si>
   <si>
     <t>Overall Cost</t>
+  </si>
+  <si>
+    <t>183</t>
+  </si>
+  <si>
+    <t>420</t>
+  </si>
+  <si>
+    <t>998917</t>
   </si>
 </sst>
 </file>
@@ -1620,23 +1629,23 @@
   <dimension ref="A1:XEO69"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14"/>
   <cols>
-    <col min="1" max="1" width="9.36363636363636" style="1" customWidth="1"/>
-    <col min="2" max="2" width="11.8181818181818" style="1" customWidth="1"/>
-    <col min="3" max="3" width="17.2727272727273" style="1" customWidth="1"/>
-    <col min="4" max="5" width="34.4545454545455" style="1" customWidth="1"/>
-    <col min="6" max="9" width="34.2727272727273" style="1" customWidth="1"/>
-    <col min="10" max="10" width="15.3636363636364" style="1" customWidth="1"/>
-    <col min="11" max="11" width="34.2727272727273" style="1" customWidth="1"/>
-    <col min="12" max="12" width="14.3636363636364" style="1" customWidth="1"/>
-    <col min="13" max="13" width="16.1818181818182" style="1" customWidth="1"/>
-    <col min="14" max="14" width="19.3636363636364" style="1" customWidth="1"/>
-    <col min="15" max="15" width="19.6363636363636" style="1" customWidth="1"/>
-    <col min="16" max="16" width="15.9090909090909" style="1" customWidth="1"/>
-    <col min="17" max="17" width="21.1818181818182" style="1" customWidth="1"/>
-    <col min="18" max="18" width="14.3636363636364" style="1" customWidth="1"/>
-    <col min="19" max="19" width="19.6363636363636" style="1" customWidth="1"/>
-    <col min="20" max="16369" width="9.13636363636364" style="1"/>
-    <col min="16370" max="16384" width="9" style="2"/>
+    <col min="1" max="1" customWidth="true" style="1" width="9.36363636363636"/>
+    <col min="2" max="2" customWidth="true" style="1" width="11.8181818181818"/>
+    <col min="3" max="3" customWidth="true" style="1" width="17.2727272727273"/>
+    <col min="4" max="5" customWidth="true" style="1" width="34.4545454545455"/>
+    <col min="6" max="9" customWidth="true" style="1" width="34.2727272727273"/>
+    <col min="10" max="10" customWidth="true" style="1" width="15.3636363636364"/>
+    <col min="11" max="11" customWidth="true" style="1" width="34.2727272727273"/>
+    <col min="12" max="12" customWidth="true" style="1" width="14.3636363636364"/>
+    <col min="13" max="13" customWidth="true" style="1" width="16.1818181818182"/>
+    <col min="14" max="14" customWidth="true" style="1" width="19.3636363636364"/>
+    <col min="15" max="15" customWidth="true" style="1" width="19.6363636363636"/>
+    <col min="16" max="16" customWidth="true" style="1" width="15.9090909090909"/>
+    <col min="17" max="17" customWidth="true" style="1" width="21.1818181818182"/>
+    <col min="18" max="18" customWidth="true" style="1" width="14.3636363636364"/>
+    <col min="19" max="19" customWidth="true" style="1" width="19.6363636363636"/>
+    <col min="20" max="16369" style="1" width="9.13636363636364"/>
+    <col min="16370" max="16384" style="2" width="9.0"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:31 16368:16369">
@@ -1724,12 +1733,16 @@
       <c r="H3" s="8">
         <v>3</v>
       </c>
-      <c r="I3" s="10"/>
+      <c r="I3" t="s" s="1">
+        <v>93</v>
+      </c>
       <c r="J3" s="10">
         <f>I3+H3</f>
         <v>3</v>
       </c>
-      <c r="K3" s="10"/>
+      <c r="K3" t="s" s="1">
+        <v>94</v>
+      </c>
       <c r="L3" s="10"/>
       <c r="M3" s="11">
         <f>L68</f>
@@ -2053,7 +2066,9 @@
       <c r="G11" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="H11" s="10"/>
+      <c r="H11" t="s" s="1">
+        <v>95</v>
+      </c>
       <c r="I11" s="10">
         <v>0</v>
       </c>
@@ -2091,7 +2106,9 @@
       <c r="G12" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="H12" s="10"/>
+      <c r="H12" t="s" s="1">
+        <v>95</v>
+      </c>
       <c r="I12" s="10">
         <v>0</v>
       </c>
@@ -2130,7 +2147,9 @@
       <c r="G13" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="H13" s="10"/>
+      <c r="H13" t="s" s="1">
+        <v>95</v>
+      </c>
       <c r="I13" s="10">
         <v>0</v>
       </c>
@@ -2169,7 +2188,9 @@
       <c r="G14" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="H14" s="10"/>
+      <c r="H14" t="s" s="1">
+        <v>95</v>
+      </c>
       <c r="I14" s="10">
         <v>0</v>
       </c>
@@ -2208,7 +2229,9 @@
       <c r="G15" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="H15" s="10"/>
+      <c r="H15" t="s" s="1">
+        <v>95</v>
+      </c>
       <c r="I15" s="10">
         <v>0</v>
       </c>
@@ -2247,7 +2270,9 @@
       <c r="G16" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="H16" s="10"/>
+      <c r="H16" t="s" s="1">
+        <v>95</v>
+      </c>
       <c r="I16" s="10">
         <v>0</v>
       </c>
@@ -2286,7 +2311,9 @@
       <c r="G17" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="H17" s="10"/>
+      <c r="H17" t="s" s="1">
+        <v>95</v>
+      </c>
       <c r="I17" s="10">
         <v>0</v>
       </c>

</xml_diff>

<commit_message>
Production order and BOM fixes
Production order and BOM fixes
</commit_message>
<xml_diff>
--- a/testdata/PMF - Scenarios.xlsx
+++ b/testdata/PMF - Scenarios.xlsx
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8458" uniqueCount="200">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9562" uniqueCount="224">
   <si>
     <t>Production Order - All Inside</t>
   </si>
@@ -641,6 +641,78 @@
   </si>
   <si>
     <t>998507</t>
+  </si>
+  <si>
+    <t>208</t>
+  </si>
+  <si>
+    <t>998487</t>
+  </si>
+  <si>
+    <t>99963</t>
+  </si>
+  <si>
+    <t>99966</t>
+  </si>
+  <si>
+    <t>998484</t>
+  </si>
+  <si>
+    <t>998481</t>
+  </si>
+  <si>
+    <t>998478</t>
+  </si>
+  <si>
+    <t>998475</t>
+  </si>
+  <si>
+    <t>998472</t>
+  </si>
+  <si>
+    <t>998469</t>
+  </si>
+  <si>
+    <t>998466</t>
+  </si>
+  <si>
+    <t>998463</t>
+  </si>
+  <si>
+    <t>99960</t>
+  </si>
+  <si>
+    <t>998460</t>
+  </si>
+  <si>
+    <t>99957</t>
+  </si>
+  <si>
+    <t>998457</t>
+  </si>
+  <si>
+    <t>998454</t>
+  </si>
+  <si>
+    <t>6</t>
+  </si>
+  <si>
+    <t>9</t>
+  </si>
+  <si>
+    <t>998451</t>
+  </si>
+  <si>
+    <t>12</t>
+  </si>
+  <si>
+    <t>15</t>
+  </si>
+  <si>
+    <t>998448</t>
+  </si>
+  <si>
+    <t>18</t>
   </si>
 </sst>
 </file>
@@ -2227,7 +2299,7 @@
         <v>3</v>
       </c>
       <c r="I3" t="s" s="1">
-        <v>164</v>
+        <v>200</v>
       </c>
       <c r="J3" s="8">
         <f>I3+H3</f>
@@ -2563,10 +2635,10 @@
         <v>68</v>
       </c>
       <c r="H11" t="s" s="1">
-        <v>193</v>
+        <v>219</v>
       </c>
       <c r="I11" t="s" s="1">
-        <v>78</v>
+        <v>221</v>
       </c>
       <c r="J11" s="8">
         <f>H11-I11</f>
@@ -2603,10 +2675,10 @@
         <v>68</v>
       </c>
       <c r="H12" t="s" s="1">
-        <v>193</v>
+        <v>219</v>
       </c>
       <c r="I12" t="s" s="1">
-        <v>78</v>
+        <v>221</v>
       </c>
       <c r="J12" s="8">
         <f>H12-I12</f>
@@ -2644,10 +2716,10 @@
         <v>68</v>
       </c>
       <c r="H13" t="s" s="1">
-        <v>193</v>
+        <v>219</v>
       </c>
       <c r="I13" t="s" s="1">
-        <v>78</v>
+        <v>221</v>
       </c>
       <c r="J13" s="8">
         <f>H13-I13</f>
@@ -2685,10 +2757,10 @@
         <v>68</v>
       </c>
       <c r="H14" t="s" s="1">
-        <v>193</v>
+        <v>219</v>
       </c>
       <c r="I14" t="s" s="1">
-        <v>78</v>
+        <v>221</v>
       </c>
       <c r="J14" s="8">
         <f>H14-I14</f>
@@ -2726,10 +2798,10 @@
         <v>68</v>
       </c>
       <c r="H15" t="s" s="1">
-        <v>193</v>
+        <v>219</v>
       </c>
       <c r="I15" t="s" s="1">
-        <v>78</v>
+        <v>221</v>
       </c>
       <c r="J15" s="8">
         <f t="shared" ref="J12:J31" si="0">H15-I15</f>
@@ -2767,10 +2839,10 @@
         <v>68</v>
       </c>
       <c r="H16" t="s" s="1">
-        <v>193</v>
+        <v>219</v>
       </c>
       <c r="I16" t="s" s="1">
-        <v>78</v>
+        <v>221</v>
       </c>
       <c r="J16" s="8">
         <f t="shared" si="0"/>
@@ -2808,10 +2880,10 @@
         <v>68</v>
       </c>
       <c r="H17" t="s" s="1">
-        <v>193</v>
+        <v>219</v>
       </c>
       <c r="I17" t="s" s="1">
-        <v>78</v>
+        <v>221</v>
       </c>
       <c r="J17" s="8">
         <f t="shared" si="0"/>
@@ -3583,7 +3655,7 @@
         <v>3</v>
       </c>
       <c r="O36" t="s" s="1">
-        <v>193</v>
+        <v>219</v>
       </c>
       <c r="P36" s="8">
         <f>O36-I36</f>
@@ -3647,7 +3719,7 @@
         <v>3</v>
       </c>
       <c r="O37" t="s" s="1">
-        <v>193</v>
+        <v>219</v>
       </c>
       <c r="P37" s="8">
         <f t="shared" ref="P37:P42" si="5">O37-I37</f>
@@ -3711,7 +3783,7 @@
         <v>3</v>
       </c>
       <c r="O38" t="s" s="1">
-        <v>193</v>
+        <v>219</v>
       </c>
       <c r="P38" s="8">
         <f t="shared" si="5"/>
@@ -3775,7 +3847,7 @@
         <v>3</v>
       </c>
       <c r="O39" t="s" s="1">
-        <v>193</v>
+        <v>219</v>
       </c>
       <c r="P39" s="8">
         <f t="shared" si="5"/>
@@ -3839,7 +3911,7 @@
         <v>3</v>
       </c>
       <c r="O40" t="s" s="1">
-        <v>193</v>
+        <v>219</v>
       </c>
       <c r="P40" s="8">
         <f t="shared" si="5"/>
@@ -3903,7 +3975,7 @@
         <v>3</v>
       </c>
       <c r="O41" t="s" s="1">
-        <v>193</v>
+        <v>219</v>
       </c>
       <c r="P41" s="8">
         <f t="shared" si="5"/>
@@ -3967,7 +4039,7 @@
         <v>3</v>
       </c>
       <c r="O42" t="s" s="1">
-        <v>193</v>
+        <v>219</v>
       </c>
       <c r="P42" s="8">
         <f t="shared" si="5"/>
@@ -4147,7 +4219,7 @@
         <v>3</v>
       </c>
       <c r="O46" t="s" s="1">
-        <v>192</v>
+        <v>214</v>
       </c>
       <c r="P46" s="8">
         <f>O46-I46</f>
@@ -4211,7 +4283,7 @@
         <v>3</v>
       </c>
       <c r="O47" t="s" s="1">
-        <v>192</v>
+        <v>214</v>
       </c>
       <c r="P47" s="8">
         <f t="shared" ref="P47:P52" si="10">O47-I47</f>
@@ -4275,7 +4347,7 @@
         <v>3</v>
       </c>
       <c r="O48" t="s" s="1">
-        <v>192</v>
+        <v>214</v>
       </c>
       <c r="P48" s="8">
         <f t="shared" si="10"/>
@@ -4339,7 +4411,7 @@
         <v>3</v>
       </c>
       <c r="O49" t="s" s="1">
-        <v>192</v>
+        <v>214</v>
       </c>
       <c r="P49" s="8">
         <f t="shared" si="10"/>
@@ -4403,7 +4475,7 @@
         <v>3</v>
       </c>
       <c r="O50" t="s" s="1">
-        <v>192</v>
+        <v>214</v>
       </c>
       <c r="P50" s="8">
         <f t="shared" si="10"/>
@@ -4467,7 +4539,7 @@
         <v>3</v>
       </c>
       <c r="O51" t="s" s="1">
-        <v>192</v>
+        <v>214</v>
       </c>
       <c r="P51" s="8">
         <f t="shared" si="10"/>
@@ -4531,7 +4603,7 @@
         <v>3</v>
       </c>
       <c r="O52" t="s" s="1">
-        <v>192</v>
+        <v>214</v>
       </c>
       <c r="P52" s="8">
         <f t="shared" si="10"/>
@@ -4761,7 +4833,7 @@
         <v>0</v>
       </c>
       <c r="O57" t="s" s="1">
-        <v>190</v>
+        <v>212</v>
       </c>
       <c r="P57" s="8">
         <f>O57-I57</f>
@@ -4825,7 +4897,7 @@
         <v>0</v>
       </c>
       <c r="O58" t="s" s="1">
-        <v>190</v>
+        <v>212</v>
       </c>
       <c r="P58" s="8">
         <f t="shared" ref="P58:P63" si="14">O58-I58</f>
@@ -4889,7 +4961,7 @@
         <v>0</v>
       </c>
       <c r="O59" t="s" s="1">
-        <v>190</v>
+        <v>212</v>
       </c>
       <c r="P59" s="8">
         <f t="shared" si="14"/>
@@ -4953,7 +5025,7 @@
         <v>0</v>
       </c>
       <c r="O60" t="s" s="1">
-        <v>190</v>
+        <v>212</v>
       </c>
       <c r="P60" s="8">
         <f t="shared" si="14"/>
@@ -5017,7 +5089,7 @@
         <v>0</v>
       </c>
       <c r="O61" t="s" s="1">
-        <v>190</v>
+        <v>212</v>
       </c>
       <c r="P61" s="8">
         <f t="shared" si="14"/>
@@ -5081,7 +5153,7 @@
         <v>0</v>
       </c>
       <c r="O62" t="s" s="1">
-        <v>190</v>
+        <v>212</v>
       </c>
       <c r="P62" s="8">
         <f t="shared" si="14"/>
@@ -5145,7 +5217,7 @@
         <v>0</v>
       </c>
       <c r="O63" t="s" s="1">
-        <v>190</v>
+        <v>212</v>
       </c>
       <c r="P63" s="8">
         <f t="shared" si="14"/>
@@ -26984,7 +27056,7 @@
         <v>3</v>
       </c>
       <c r="I3" t="s" s="1">
-        <v>164</v>
+        <v>200</v>
       </c>
       <c r="J3" s="8">
         <f>I3+H3</f>
@@ -27320,10 +27392,10 @@
         <v>68</v>
       </c>
       <c r="H11" t="s" s="1">
-        <v>195</v>
+        <v>222</v>
       </c>
       <c r="I11" t="s" s="1">
-        <v>78</v>
+        <v>220</v>
       </c>
       <c r="J11" s="8">
         <f t="shared" ref="J11:J31" si="0">H11-I11</f>
@@ -27360,10 +27432,10 @@
         <v>68</v>
       </c>
       <c r="H12" t="s" s="1">
-        <v>195</v>
+        <v>222</v>
       </c>
       <c r="I12" t="s" s="1">
-        <v>78</v>
+        <v>220</v>
       </c>
       <c r="J12" s="8">
         <f t="shared" si="0"/>
@@ -27401,10 +27473,10 @@
         <v>68</v>
       </c>
       <c r="H13" t="s" s="1">
-        <v>195</v>
+        <v>222</v>
       </c>
       <c r="I13" t="s" s="1">
-        <v>78</v>
+        <v>220</v>
       </c>
       <c r="J13" s="8">
         <f t="shared" si="0"/>
@@ -27442,10 +27514,10 @@
         <v>68</v>
       </c>
       <c r="H14" t="s" s="1">
-        <v>195</v>
+        <v>222</v>
       </c>
       <c r="I14" t="s" s="1">
-        <v>78</v>
+        <v>220</v>
       </c>
       <c r="J14" s="8">
         <f t="shared" si="0"/>
@@ -27483,10 +27555,10 @@
         <v>68</v>
       </c>
       <c r="H15" t="s" s="1">
-        <v>195</v>
+        <v>222</v>
       </c>
       <c r="I15" t="s" s="1">
-        <v>78</v>
+        <v>220</v>
       </c>
       <c r="J15" s="8">
         <f t="shared" si="0"/>
@@ -27524,10 +27596,10 @@
         <v>68</v>
       </c>
       <c r="H16" t="s" s="1">
-        <v>195</v>
+        <v>222</v>
       </c>
       <c r="I16" t="s" s="1">
-        <v>78</v>
+        <v>220</v>
       </c>
       <c r="J16" s="8">
         <f t="shared" si="0"/>
@@ -27565,10 +27637,10 @@
         <v>68</v>
       </c>
       <c r="H17" t="s" s="1">
-        <v>195</v>
+        <v>222</v>
       </c>
       <c r="I17" t="s" s="1">
-        <v>78</v>
+        <v>220</v>
       </c>
       <c r="J17" s="8">
         <f t="shared" si="0"/>
@@ -28340,7 +28412,7 @@
         <v>3</v>
       </c>
       <c r="O36" t="s" s="1">
-        <v>195</v>
+        <v>222</v>
       </c>
       <c r="P36" s="8">
         <f t="shared" ref="P36:P42" si="4">O36-I36</f>
@@ -28404,7 +28476,7 @@
         <v>3</v>
       </c>
       <c r="O37" t="s" s="1">
-        <v>195</v>
+        <v>222</v>
       </c>
       <c r="P37" s="8">
         <f t="shared" si="4"/>
@@ -28468,7 +28540,7 @@
         <v>3</v>
       </c>
       <c r="O38" t="s" s="1">
-        <v>195</v>
+        <v>222</v>
       </c>
       <c r="P38" s="8">
         <f t="shared" si="4"/>
@@ -28532,7 +28604,7 @@
         <v>3</v>
       </c>
       <c r="O39" t="s" s="1">
-        <v>195</v>
+        <v>222</v>
       </c>
       <c r="P39" s="8">
         <f t="shared" si="4"/>
@@ -28596,7 +28668,7 @@
         <v>3</v>
       </c>
       <c r="O40" t="s" s="1">
-        <v>195</v>
+        <v>222</v>
       </c>
       <c r="P40" s="8">
         <f t="shared" si="4"/>
@@ -28660,7 +28732,7 @@
         <v>3</v>
       </c>
       <c r="O41" t="s" s="1">
-        <v>195</v>
+        <v>222</v>
       </c>
       <c r="P41" s="8">
         <f t="shared" si="4"/>
@@ -28724,7 +28796,7 @@
         <v>3</v>
       </c>
       <c r="O42" t="s" s="1">
-        <v>195</v>
+        <v>222</v>
       </c>
       <c r="P42" s="8">
         <f t="shared" si="4"/>
@@ -28904,7 +28976,7 @@
         <v>3</v>
       </c>
       <c r="O46" t="s" s="1">
-        <v>192</v>
+        <v>214</v>
       </c>
       <c r="P46" s="8">
         <f t="shared" ref="P46:P52" si="9">O46-I46</f>
@@ -28968,7 +29040,7 @@
         <v>3</v>
       </c>
       <c r="O47" t="s" s="1">
-        <v>192</v>
+        <v>214</v>
       </c>
       <c r="P47" s="8">
         <f t="shared" si="9"/>
@@ -29032,7 +29104,7 @@
         <v>3</v>
       </c>
       <c r="O48" t="s" s="1">
-        <v>192</v>
+        <v>214</v>
       </c>
       <c r="P48" s="8">
         <f t="shared" si="9"/>
@@ -29096,7 +29168,7 @@
         <v>3</v>
       </c>
       <c r="O49" t="s" s="1">
-        <v>192</v>
+        <v>214</v>
       </c>
       <c r="P49" s="8">
         <f t="shared" si="9"/>
@@ -29160,7 +29232,7 @@
         <v>3</v>
       </c>
       <c r="O50" t="s" s="1">
-        <v>192</v>
+        <v>214</v>
       </c>
       <c r="P50" s="8">
         <f t="shared" si="9"/>
@@ -29224,7 +29296,7 @@
         <v>3</v>
       </c>
       <c r="O51" t="s" s="1">
-        <v>192</v>
+        <v>214</v>
       </c>
       <c r="P51" s="8">
         <f t="shared" si="9"/>
@@ -29288,7 +29360,7 @@
         <v>3</v>
       </c>
       <c r="O52" t="s" s="1">
-        <v>192</v>
+        <v>214</v>
       </c>
       <c r="P52" s="8">
         <f t="shared" si="9"/>
@@ -29352,7 +29424,7 @@
         <v>3</v>
       </c>
       <c r="O53" t="s" s="1">
-        <v>190</v>
+        <v>212</v>
       </c>
       <c r="P53" s="8">
         <f t="shared" ref="P53:P59" si="14">O53-I53</f>
@@ -29416,7 +29488,7 @@
         <v>3</v>
       </c>
       <c r="O54" t="s" s="1">
-        <v>190</v>
+        <v>212</v>
       </c>
       <c r="P54" s="8">
         <f t="shared" si="14"/>
@@ -29480,7 +29552,7 @@
         <v>3</v>
       </c>
       <c r="O55" t="s" s="1">
-        <v>190</v>
+        <v>212</v>
       </c>
       <c r="P55" s="8">
         <f t="shared" si="14"/>
@@ -29544,7 +29616,7 @@
         <v>3</v>
       </c>
       <c r="O56" t="s" s="1">
-        <v>190</v>
+        <v>212</v>
       </c>
       <c r="P56" s="8">
         <f t="shared" si="14"/>
@@ -29608,7 +29680,7 @@
         <v>3</v>
       </c>
       <c r="O57" t="s" s="1">
-        <v>190</v>
+        <v>212</v>
       </c>
       <c r="P57" s="8">
         <f t="shared" si="14"/>
@@ -29672,7 +29744,7 @@
         <v>3</v>
       </c>
       <c r="O58" t="s" s="1">
-        <v>190</v>
+        <v>212</v>
       </c>
       <c r="P58" s="8">
         <f t="shared" si="14"/>
@@ -29736,7 +29808,7 @@
         <v>3</v>
       </c>
       <c r="O59" t="s" s="1">
-        <v>190</v>
+        <v>212</v>
       </c>
       <c r="P59" s="8">
         <f t="shared" si="14"/>
@@ -30057,7 +30129,7 @@
         <v>3</v>
       </c>
       <c r="I3" t="s" s="1">
-        <v>164</v>
+        <v>200</v>
       </c>
       <c r="J3" s="8">
         <f>I3+H3</f>
@@ -30393,10 +30465,10 @@
         <v>68</v>
       </c>
       <c r="H11" t="s" s="1">
-        <v>197</v>
+        <v>222</v>
       </c>
       <c r="I11" t="s" s="1">
-        <v>78</v>
+        <v>221</v>
       </c>
       <c r="J11" s="8">
         <f t="shared" ref="J11:J31" si="0">H11-I11</f>
@@ -30433,10 +30505,10 @@
         <v>68</v>
       </c>
       <c r="H12" t="s" s="1">
-        <v>197</v>
+        <v>222</v>
       </c>
       <c r="I12" t="s" s="1">
-        <v>78</v>
+        <v>221</v>
       </c>
       <c r="J12" s="8">
         <f t="shared" si="0"/>
@@ -30474,10 +30546,10 @@
         <v>68</v>
       </c>
       <c r="H13" t="s" s="1">
-        <v>197</v>
+        <v>222</v>
       </c>
       <c r="I13" t="s" s="1">
-        <v>78</v>
+        <v>221</v>
       </c>
       <c r="J13" s="8">
         <f t="shared" si="0"/>
@@ -30515,10 +30587,10 @@
         <v>68</v>
       </c>
       <c r="H14" t="s" s="1">
-        <v>197</v>
+        <v>222</v>
       </c>
       <c r="I14" t="s" s="1">
-        <v>78</v>
+        <v>221</v>
       </c>
       <c r="J14" s="8">
         <f t="shared" si="0"/>
@@ -30556,10 +30628,10 @@
         <v>68</v>
       </c>
       <c r="H15" t="s" s="1">
-        <v>197</v>
+        <v>222</v>
       </c>
       <c r="I15" t="s" s="1">
-        <v>78</v>
+        <v>221</v>
       </c>
       <c r="J15" s="8">
         <f t="shared" si="0"/>
@@ -30597,10 +30669,10 @@
         <v>68</v>
       </c>
       <c r="H16" t="s" s="1">
-        <v>197</v>
+        <v>222</v>
       </c>
       <c r="I16" t="s" s="1">
-        <v>78</v>
+        <v>221</v>
       </c>
       <c r="J16" s="8">
         <f t="shared" si="0"/>
@@ -30638,10 +30710,10 @@
         <v>68</v>
       </c>
       <c r="H17" t="s" s="1">
-        <v>197</v>
+        <v>222</v>
       </c>
       <c r="I17" t="s" s="1">
-        <v>78</v>
+        <v>221</v>
       </c>
       <c r="J17" s="8">
         <f t="shared" si="0"/>
@@ -31413,7 +31485,7 @@
         <v>3</v>
       </c>
       <c r="O36" t="s" s="1">
-        <v>197</v>
+        <v>222</v>
       </c>
       <c r="P36" s="8">
         <f t="shared" ref="P36:P42" si="4">O36-I36</f>
@@ -31477,7 +31549,7 @@
         <v>3</v>
       </c>
       <c r="O37" t="s" s="1">
-        <v>197</v>
+        <v>222</v>
       </c>
       <c r="P37" s="8">
         <f t="shared" si="4"/>
@@ -31541,7 +31613,7 @@
         <v>3</v>
       </c>
       <c r="O38" t="s" s="1">
-        <v>197</v>
+        <v>222</v>
       </c>
       <c r="P38" s="8">
         <f t="shared" si="4"/>
@@ -31605,7 +31677,7 @@
         <v>3</v>
       </c>
       <c r="O39" t="s" s="1">
-        <v>197</v>
+        <v>222</v>
       </c>
       <c r="P39" s="8">
         <f t="shared" si="4"/>
@@ -31669,7 +31741,7 @@
         <v>3</v>
       </c>
       <c r="O40" t="s" s="1">
-        <v>197</v>
+        <v>222</v>
       </c>
       <c r="P40" s="8">
         <f t="shared" si="4"/>
@@ -31733,7 +31805,7 @@
         <v>3</v>
       </c>
       <c r="O41" t="s" s="1">
-        <v>197</v>
+        <v>222</v>
       </c>
       <c r="P41" s="8">
         <f t="shared" si="4"/>
@@ -31797,7 +31869,7 @@
         <v>3</v>
       </c>
       <c r="O42" t="s" s="1">
-        <v>197</v>
+        <v>222</v>
       </c>
       <c r="P42" s="8">
         <f t="shared" si="4"/>
@@ -31861,7 +31933,7 @@
         <v>3</v>
       </c>
       <c r="O43" t="s" s="1">
-        <v>198</v>
+        <v>214</v>
       </c>
       <c r="P43" s="8">
         <f t="shared" ref="P43:P56" si="9">O43-I43</f>
@@ -31925,7 +31997,7 @@
         <v>3</v>
       </c>
       <c r="O44" t="s" s="1">
-        <v>198</v>
+        <v>214</v>
       </c>
       <c r="P44" s="8">
         <f t="shared" si="9"/>
@@ -31989,7 +32061,7 @@
         <v>3</v>
       </c>
       <c r="O45" t="s" s="1">
-        <v>198</v>
+        <v>214</v>
       </c>
       <c r="P45" s="8">
         <f t="shared" si="9"/>
@@ -32053,7 +32125,7 @@
         <v>3</v>
       </c>
       <c r="O46" t="s" s="1">
-        <v>198</v>
+        <v>214</v>
       </c>
       <c r="P46" s="8">
         <f t="shared" si="9"/>
@@ -32117,7 +32189,7 @@
         <v>3</v>
       </c>
       <c r="O47" t="s" s="1">
-        <v>198</v>
+        <v>214</v>
       </c>
       <c r="P47" s="8">
         <f t="shared" si="9"/>
@@ -32181,7 +32253,7 @@
         <v>3</v>
       </c>
       <c r="O48" t="s" s="1">
-        <v>198</v>
+        <v>214</v>
       </c>
       <c r="P48" s="8">
         <f t="shared" si="9"/>
@@ -32245,7 +32317,7 @@
         <v>3</v>
       </c>
       <c r="O49" t="s" s="1">
-        <v>198</v>
+        <v>214</v>
       </c>
       <c r="P49" s="8">
         <f t="shared" si="9"/>
@@ -32309,7 +32381,7 @@
         <v>3</v>
       </c>
       <c r="O50" t="s" s="1">
-        <v>192</v>
+        <v>212</v>
       </c>
       <c r="P50" s="8">
         <f t="shared" si="9"/>
@@ -32373,7 +32445,7 @@
         <v>3</v>
       </c>
       <c r="O51" t="s" s="1">
-        <v>192</v>
+        <v>212</v>
       </c>
       <c r="P51" s="8">
         <f t="shared" si="9"/>
@@ -32437,7 +32509,7 @@
         <v>3</v>
       </c>
       <c r="O52" t="s" s="1">
-        <v>192</v>
+        <v>212</v>
       </c>
       <c r="P52" s="8">
         <f t="shared" si="9"/>
@@ -32501,7 +32573,7 @@
         <v>3</v>
       </c>
       <c r="O53" t="s" s="1">
-        <v>192</v>
+        <v>212</v>
       </c>
       <c r="P53" s="8">
         <f t="shared" si="9"/>
@@ -32565,7 +32637,7 @@
         <v>3</v>
       </c>
       <c r="O54" t="s" s="1">
-        <v>192</v>
+        <v>212</v>
       </c>
       <c r="P54" s="8">
         <f t="shared" si="9"/>
@@ -32629,7 +32701,7 @@
         <v>3</v>
       </c>
       <c r="O55" t="s" s="1">
-        <v>192</v>
+        <v>212</v>
       </c>
       <c r="P55" s="8">
         <f t="shared" si="9"/>
@@ -32693,7 +32765,7 @@
         <v>3</v>
       </c>
       <c r="O56" t="s" s="1">
-        <v>192</v>
+        <v>212</v>
       </c>
       <c r="P56" s="8">
         <f t="shared" si="9"/>
@@ -33040,7 +33112,7 @@
         <v>3</v>
       </c>
       <c r="I3" t="s" s="1">
-        <v>164</v>
+        <v>200</v>
       </c>
       <c r="J3" s="8">
         <f>I3+H3</f>
@@ -33371,10 +33443,10 @@
         <v>68</v>
       </c>
       <c r="H11" t="s" s="1">
-        <v>199</v>
+        <v>222</v>
       </c>
       <c r="I11" t="s" s="1">
-        <v>70</v>
+        <v>223</v>
       </c>
       <c r="J11" s="8">
         <f t="shared" ref="J11:J31" si="0">H11-I11</f>
@@ -33412,10 +33484,10 @@
         <v>68</v>
       </c>
       <c r="H12" t="s" s="1">
-        <v>199</v>
+        <v>222</v>
       </c>
       <c r="I12" t="s" s="1">
-        <v>70</v>
+        <v>223</v>
       </c>
       <c r="J12" s="8">
         <f t="shared" si="0"/>
@@ -33453,10 +33525,10 @@
         <v>68</v>
       </c>
       <c r="H13" t="s" s="1">
-        <v>199</v>
+        <v>222</v>
       </c>
       <c r="I13" t="s" s="1">
-        <v>70</v>
+        <v>223</v>
       </c>
       <c r="J13" s="8">
         <f t="shared" si="0"/>
@@ -33494,10 +33566,10 @@
         <v>68</v>
       </c>
       <c r="H14" t="s" s="1">
-        <v>199</v>
+        <v>222</v>
       </c>
       <c r="I14" t="s" s="1">
-        <v>70</v>
+        <v>223</v>
       </c>
       <c r="J14" s="8">
         <f t="shared" si="0"/>
@@ -33535,10 +33607,10 @@
         <v>68</v>
       </c>
       <c r="H15" t="s" s="1">
-        <v>199</v>
+        <v>222</v>
       </c>
       <c r="I15" t="s" s="1">
-        <v>70</v>
+        <v>223</v>
       </c>
       <c r="J15" s="8">
         <f t="shared" si="0"/>
@@ -33576,10 +33648,10 @@
         <v>68</v>
       </c>
       <c r="H16" t="s" s="1">
-        <v>199</v>
+        <v>222</v>
       </c>
       <c r="I16" t="s" s="1">
-        <v>70</v>
+        <v>223</v>
       </c>
       <c r="J16" s="8">
         <f t="shared" si="0"/>
@@ -33617,10 +33689,10 @@
         <v>68</v>
       </c>
       <c r="H17" t="s" s="1">
-        <v>199</v>
+        <v>222</v>
       </c>
       <c r="I17" t="s" s="1">
-        <v>70</v>
+        <v>223</v>
       </c>
       <c r="J17" s="8">
         <f t="shared" si="0"/>
@@ -37169,7 +37241,7 @@
         <v>3</v>
       </c>
       <c r="I3" t="s" s="1">
-        <v>164</v>
+        <v>200</v>
       </c>
       <c r="J3" s="8">
         <f>I3+H3</f>
@@ -37500,10 +37572,10 @@
         <v>68</v>
       </c>
       <c r="H11" t="s" s="1">
-        <v>199</v>
+        <v>222</v>
       </c>
       <c r="I11" t="s" s="1">
-        <v>70</v>
+        <v>223</v>
       </c>
       <c r="J11" s="8">
         <f t="shared" ref="J11:J31" si="0">H11-I11</f>
@@ -37541,10 +37613,10 @@
         <v>68</v>
       </c>
       <c r="H12" t="s" s="1">
-        <v>199</v>
+        <v>222</v>
       </c>
       <c r="I12" t="s" s="1">
-        <v>70</v>
+        <v>223</v>
       </c>
       <c r="J12" s="8">
         <f t="shared" si="0"/>
@@ -37582,10 +37654,10 @@
         <v>68</v>
       </c>
       <c r="H13" t="s" s="1">
-        <v>199</v>
+        <v>222</v>
       </c>
       <c r="I13" t="s" s="1">
-        <v>70</v>
+        <v>223</v>
       </c>
       <c r="J13" s="8">
         <f t="shared" si="0"/>
@@ -37623,10 +37695,10 @@
         <v>68</v>
       </c>
       <c r="H14" t="s" s="1">
-        <v>199</v>
+        <v>222</v>
       </c>
       <c r="I14" t="s" s="1">
-        <v>70</v>
+        <v>223</v>
       </c>
       <c r="J14" s="8">
         <f t="shared" si="0"/>
@@ -37664,10 +37736,10 @@
         <v>68</v>
       </c>
       <c r="H15" t="s" s="1">
-        <v>199</v>
+        <v>222</v>
       </c>
       <c r="I15" t="s" s="1">
-        <v>70</v>
+        <v>223</v>
       </c>
       <c r="J15" s="8">
         <f t="shared" si="0"/>
@@ -37705,10 +37777,10 @@
         <v>68</v>
       </c>
       <c r="H16" t="s" s="1">
-        <v>199</v>
+        <v>222</v>
       </c>
       <c r="I16" t="s" s="1">
-        <v>70</v>
+        <v>223</v>
       </c>
       <c r="J16" s="8">
         <f t="shared" si="0"/>
@@ -37746,10 +37818,10 @@
         <v>68</v>
       </c>
       <c r="H17" t="s" s="1">
-        <v>199</v>
+        <v>222</v>
       </c>
       <c r="I17" t="s" s="1">
-        <v>70</v>
+        <v>223</v>
       </c>
       <c r="J17" s="8">
         <f t="shared" si="0"/>
@@ -40993,7 +41065,7 @@
         <v>3</v>
       </c>
       <c r="I3" t="s" s="1">
-        <v>164</v>
+        <v>200</v>
       </c>
       <c r="J3" s="8">
         <f>I3+H3</f>
@@ -41324,10 +41396,10 @@
         <v>68</v>
       </c>
       <c r="H11" t="s" s="1">
-        <v>199</v>
+        <v>222</v>
       </c>
       <c r="I11" t="s" s="1">
-        <v>70</v>
+        <v>223</v>
       </c>
       <c r="J11" s="8">
         <f t="shared" ref="J11:J31" si="0">H11-I11</f>
@@ -41365,10 +41437,10 @@
         <v>68</v>
       </c>
       <c r="H12" t="s" s="1">
-        <v>199</v>
+        <v>222</v>
       </c>
       <c r="I12" t="s" s="1">
-        <v>70</v>
+        <v>223</v>
       </c>
       <c r="J12" s="8">
         <f t="shared" si="0"/>
@@ -41406,10 +41478,10 @@
         <v>68</v>
       </c>
       <c r="H13" t="s" s="1">
-        <v>199</v>
+        <v>222</v>
       </c>
       <c r="I13" t="s" s="1">
-        <v>70</v>
+        <v>223</v>
       </c>
       <c r="J13" s="8">
         <f t="shared" si="0"/>
@@ -41447,10 +41519,10 @@
         <v>68</v>
       </c>
       <c r="H14" t="s" s="1">
-        <v>199</v>
+        <v>222</v>
       </c>
       <c r="I14" t="s" s="1">
-        <v>70</v>
+        <v>223</v>
       </c>
       <c r="J14" s="8">
         <f t="shared" si="0"/>
@@ -41488,10 +41560,10 @@
         <v>68</v>
       </c>
       <c r="H15" t="s" s="1">
-        <v>199</v>
+        <v>222</v>
       </c>
       <c r="I15" t="s" s="1">
-        <v>70</v>
+        <v>223</v>
       </c>
       <c r="J15" s="8">
         <f t="shared" si="0"/>
@@ -41529,10 +41601,10 @@
         <v>68</v>
       </c>
       <c r="H16" t="s" s="1">
-        <v>199</v>
+        <v>222</v>
       </c>
       <c r="I16" t="s" s="1">
-        <v>70</v>
+        <v>223</v>
       </c>
       <c r="J16" s="8">
         <f t="shared" si="0"/>
@@ -41570,10 +41642,10 @@
         <v>68</v>
       </c>
       <c r="H17" t="s" s="1">
-        <v>199</v>
+        <v>222</v>
       </c>
       <c r="I17" t="s" s="1">
-        <v>70</v>
+        <v>223</v>
       </c>
       <c r="J17" s="8">
         <f t="shared" si="0"/>

</xml_diff>